<commit_message>
Fix unused variable TS errors and update player data
</commit_message>
<xml_diff>
--- a/backend/playerdata.xlsx
+++ b/backend/playerdata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -807,10 +807,8 @@
           <t>Soumo Bro</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="C19" t="n">
+        <v>123</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
@@ -830,13 +828,57 @@
           <t>Soumya</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="C20" t="n">
+        <v>123</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Swarnadeep</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Swarna</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Shounak</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Shounak</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
         <is>
           <t>player</t>
         </is>

</xml_diff>